<commit_message>
feat & fix: JSON 反向转 Excel 工具与校验修复
- 新增 json_to_excel.py，支持卡牌/遗物/事件 JSON 批量回写 Excel
- 更新 cards.xlsx / artifacts.xlsx / events.xlsx 与当前 JSON 数据同步
- 修复 excel_to_json.py 中卡牌 target 校验逻辑：
  允许 AoE（target_override=ALL_ENEMIES）攻击牌设置 requires_target=false
</commit_message>
<xml_diff>
--- a/external/config/artifacts.xlsx
+++ b/external/config/artifacts.xlsx
@@ -435,15 +435,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:AE24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="47" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
@@ -453,11 +453,22 @@
     <col width="36" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="34" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="29" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="17" max="17"/>
+    <col width="33" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="31" customWidth="1" min="20" max="20"/>
+    <col width="32" customWidth="1" min="21" max="21"/>
+    <col width="33" customWidth="1" min="22" max="22"/>
+    <col width="34" customWidth="1" min="23" max="23"/>
+    <col width="36" customWidth="1" min="24" max="24"/>
+    <col width="37" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="26" max="26"/>
+    <col width="35" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="28" max="28"/>
+    <col width="34" customWidth="1" min="29" max="29"/>
+    <col width="35" customWidth="1" min="30" max="30"/>
+    <col width="37" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,27 +549,82 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>artifact_remove_action_type</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_remove_action_money_amount</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>artifact_turn_start_action_type</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>artifact_turn_start_action_block</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_turn_end_action_type</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_turn_end_action_block</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_first_turn_action_type</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_first_turn_action_block</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_end_of_combat_action_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_end_of_combat_action_block</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>artifact_max_counter_action_type</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>artifact_max_counter_action_block</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_max_counter_action_money_amount</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>artifact_right_click_action_type</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_right_click_action_block</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>artifact_right_click_validator_type</t>
         </is>
       </c>
     </row>
@@ -595,6 +661,17 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -661,6 +738,21 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -718,15 +810,1562 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>ActionBlock</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="AA4" t="n">
         <v>5</v>
       </c>
-      <c r="T4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>artifact_boss_blue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Artifact Blue Boss</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Test Blue Boss Artifact.</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_blue.png</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>artifact_boss_green</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Artifact Green Boss</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Test Green Boss Artifact.</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_green.png</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>artifact_boss_orange</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Artifact Orange Boss</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Test Orange Boss Artifact.</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_orange.png</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>artifact_boss_red</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Artifact Red Boss</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Test Red Boss Artifact.</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>color_red</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_red.png</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>artifact_boss_white</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Artifact White Boss</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Test White Boss Artifact.</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>artifact_draw_on_combat_start</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Artifact Draw on Combat</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Draws 2 extra cards on the first turn</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_green.png</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>ActionDrawGenerator</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>artifact_draw_on_kill</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Artifact Draw on Kill</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Draws a card when an enemy is killed</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/ArtifactDrawOnKill.gd</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>artifact_easy_mode</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Artifact Easy Mode</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sets enemy HP to 1</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/ArtifactEasyMode.gd</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>999</v>
+      </c>
+      <c r="I12" t="n">
+        <v>999</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>artifact_full_heal</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Artifact Full Heal</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fully heals player when obtained</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="b">
+        <v>1</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>ActionHealPercent</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>artifact_heal_on_combat_ended</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Artifact Heal On Combat End</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Grants 5 health when combat is over</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="b">
+        <v>1</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>ActionAddHealth</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>artifact_increase_attack_on_rest</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Artifact Increase Attack on Rest</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Allows a permanent attack boost at rest sites</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_orange.png</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>ActionUpdateRestActions</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>ActionApplyStatus</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>artifact_retain_hand</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Artifact Retain Hand</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cards will be retained end of turn</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/ArtifactRetainHand.gd</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="b">
+        <v>1</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>artifact_right_click_shuffle_deck</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Artifact Reshuffle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Right click to shuffle discard into draw pile.</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_green.png</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>ActionReshuffle</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>artifact_see_top_of_draw_pile</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Artifact See Draw Pile</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>See the top cards in your draw pile</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_blue.png</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="b">
+        <v>1</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>ActionCustomUI</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>artifact_shop_blue</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Artifact Blue Shop</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Test Blue Shop Artifact.</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_blue.png</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>artifact_shop_green</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Artifact Green Shop</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Test Green Shop Artifact.</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_green.png</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>artifact_shop_orange</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Artifact Orange Shop</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Test Orange Shop Artifact.</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_orange.png</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="b">
+        <v>1</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>artifact_shop_red</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Artifact Red Shop</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Test Red Shop Artifact.</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>color_red</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_red.png</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>artifact_shop_white</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Artifact White Shop</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Test White Shop Artifact.</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="b">
+        <v>1</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>artifact_top_deck_attack_card</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Artifact Make Attack Card Innate</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Select an attack card to make appear at the top of your deck.</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>color_white</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>external/sprites/artifacts/artifact_white.png</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>res://scripts/artifacts/BaseArtifact.gd</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>ValidatorPlayerTurn</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Localize text and stabilize font rendering
</commit_message>
<xml_diff>
--- a/external/config/artifacts.xlsx
+++ b/external/config/artifacts.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Artifacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE24"/>
+  <dimension ref="A1:AF24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -547,82 +547,87 @@
           <t>artifact_add_action_money_amount</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>artifact_add_action_card_pick_text</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>artifact_remove_action_type</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>artifact_remove_action_money_amount</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>artifact_turn_start_action_type</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>artifact_turn_start_action_block</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>artifact_turn_end_action_type</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>artifact_turn_end_action_block</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>artifact_first_turn_action_type</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>artifact_first_turn_action_block</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>artifact_end_of_combat_action_type</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>artifact_end_of_combat_action_block</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>artifact_max_counter_action_type</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>artifact_max_counter_action_block</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>artifact_max_counter_action_money_amount</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>artifact_right_click_action_type</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>artifact_right_click_action_block</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>artifact_right_click_validator_type</t>
         </is>
@@ -644,34 +649,7 @@
           <t>artifact_rarity: 0=初始,1=普通,2=稀有,3=罕见,4=Boss,5=特殊 | artifact_color_id: color_white/red/green/blue/purple/orange/yellow</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -681,12 +659,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Add Money</t>
+          <t>获得金币</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Adds money when obtained</t>
+          <t>获得时提供金币</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -734,21 +712,7 @@
         <v>200</v>
       </c>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -762,12 +726,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Block on Attacks</t>
+          <t>攻击格挡</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Grants 5 block every 3 attacks</t>
+          <t>每进行3次攻击获得5点格挡</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -806,30 +770,16 @@
       <c r="M4" t="b">
         <v>1</v>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>ActionBlock</t>
         </is>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>5</v>
       </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -843,12 +793,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Artifact Blue Boss</t>
+          <t>蓝色Boss遗物</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Test Blue Boss Artifact.</t>
+          <t>测试蓝色Boss遗物。</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -887,24 +837,8 @@
       <c r="M5" t="b">
         <v>1</v>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -918,12 +852,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Artifact Green Boss</t>
+          <t>绿色Boss遗物</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Test Green Boss Artifact.</t>
+          <t>测试绿色Boss遗物。</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -962,24 +896,8 @@
       <c r="M6" t="b">
         <v>1</v>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -993,12 +911,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Artifact Orange Boss</t>
+          <t>橙色Boss遗物</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Test Orange Boss Artifact.</t>
+          <t>测试橙色Boss遗物。</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1037,24 +955,8 @@
       <c r="M7" t="b">
         <v>1</v>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1068,12 +970,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Artifact Red Boss</t>
+          <t>红色Boss遗物</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Test Red Boss Artifact.</t>
+          <t>测试红色Boss遗物。</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1112,24 +1014,8 @@
       <c r="M8" t="b">
         <v>1</v>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr">
+      <c r="AF8" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1143,12 +1029,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Artifact White Boss</t>
+          <t>白色Boss遗物</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Test White Boss Artifact.</t>
+          <t>测试白色Boss遗物。</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1187,24 +1073,8 @@
       <c r="M9" t="b">
         <v>1</v>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr">
+      <c r="AF9" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1218,12 +1088,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Artifact Draw on Combat</t>
+          <t>战斗首回合抽牌</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Draws 2 extra cards on the first turn</t>
+          <t>首回合额外抽2张牌</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1262,28 +1132,13 @@
       <c r="M10" t="b">
         <v>1</v>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>ActionDrawGenerator</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr">
+      <c r="AF10" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1297,12 +1152,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Artifact Draw on Kill</t>
+          <t>击杀抽牌</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Draws a card when an enemy is killed</t>
+          <t>击杀敌人时抽1张牌</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1341,24 +1196,8 @@
       <c r="M11" t="b">
         <v>1</v>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr">
+      <c r="AF11" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1372,12 +1211,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Artifact Easy Mode</t>
+          <t>简易模式</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sets enemy HP to 1</t>
+          <t>将敌人生命设为1</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1416,24 +1255,8 @@
       <c r="M12" t="b">
         <v>1</v>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr">
+      <c r="AF12" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1447,12 +1270,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Artifact Full Heal</t>
+          <t>完全治疗</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fully heals player when obtained</t>
+          <t>获得时将玩家完全治疗</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1496,23 +1319,8 @@
           <t>ActionHealPercent</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr">
+      <c r="AF13" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1526,12 +1334,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Artifact Heal On Combat End</t>
+          <t>战斗结束治疗</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grants 5 health when combat is over</t>
+          <t>战斗结束时获得5点生命</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1570,28 +1378,13 @@
       <c r="M14" t="b">
         <v>1</v>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>ActionAddHealth</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr">
+      <c r="AF14" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1605,12 +1398,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Artifact Increase Attack on Rest</t>
+          <t>休息强化攻击</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Allows a permanent attack boost at rest sites</t>
+          <t>在休息点永久提升攻击</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1654,27 +1447,13 @@
           <t>ActionUpdateRestActions</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>ActionApplyStatus</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr">
+      <c r="AF15" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1688,12 +1467,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Artifact Retain Hand</t>
+          <t>手牌保留</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cards will be retained end of turn</t>
+          <t>回合结束时手牌保留</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1732,24 +1511,8 @@
       <c r="M16" t="b">
         <v>1</v>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1763,12 +1526,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Artifact Reshuffle</t>
+          <t>洗牌重置</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Right click to shuffle discard into draw pile.</t>
+          <t>右键将弃牌堆洗回抽牌堆。</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1807,28 +1570,13 @@
       <c r="M17" t="b">
         <v>1</v>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>ActionReshuffle</t>
         </is>
       </c>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr">
+      <c r="AF17" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1842,12 +1590,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Artifact See Draw Pile</t>
+          <t>查看抽牌堆</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>See the top cards in your draw pile</t>
+          <t>查看抽牌堆顶的牌</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1886,28 +1634,13 @@
       <c r="M18" t="b">
         <v>1</v>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>ActionCustomUI</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr">
+      <c r="AF18" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1921,12 +1654,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Artifact Blue Shop</t>
+          <t>蓝色商店遗物</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Test Blue Shop Artifact.</t>
+          <t>测试蓝色商店遗物。</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1965,24 +1698,8 @@
       <c r="M19" t="b">
         <v>1</v>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr">
+      <c r="AF19" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -1996,12 +1713,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Artifact Green Shop</t>
+          <t>绿色商店遗物</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Test Green Shop Artifact.</t>
+          <t>测试绿色商店遗物。</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -2040,24 +1757,8 @@
       <c r="M20" t="b">
         <v>1</v>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr">
+      <c r="AF20" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -2071,12 +1772,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Artifact Orange Shop</t>
+          <t>橙色商店遗物</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Test Orange Shop Artifact.</t>
+          <t>测试橙色商店遗物。</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -2115,24 +1816,8 @@
       <c r="M21" t="b">
         <v>1</v>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr">
+      <c r="AF21" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -2146,12 +1831,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Artifact Red Shop</t>
+          <t>红色商店遗物</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Test Red Shop Artifact.</t>
+          <t>测试红色商店遗物。</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -2190,24 +1875,8 @@
       <c r="M22" t="b">
         <v>1</v>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr">
+      <c r="AF22" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -2221,12 +1890,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Artifact White Shop</t>
+          <t>白色商店遗物</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Test White Shop Artifact.</t>
+          <t>测试白色商店遗物。</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2265,24 +1934,8 @@
       <c r="M23" t="b">
         <v>1</v>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr">
+      <c r="AF23" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>
@@ -2296,12 +1949,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Artifact Make Attack Card Innate</t>
+          <t>使攻击牌置顶</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Select an attack card to make appear at the top of your deck.</t>
+          <t>选择一张攻击牌，使其显示在牌库顶端。</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2345,23 +1998,12 @@
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr">
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>选择一张牌置于牌库顶端</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
         <is>
           <t>ValidatorPlayerTurn</t>
         </is>

</xml_diff>